<commit_message>
Corrige campos de texto para uso no celular
</commit_message>
<xml_diff>
--- a/planilha_registro_atendimentos.xlsx
+++ b/planilha_registro_atendimentos.xlsx
@@ -140,7 +140,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -149,7 +149,7 @@
     <xf numFmtId="1" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">

</xml_diff>

<commit_message>
Reforca destaque vermelho para deficit
</commit_message>
<xml_diff>
--- a/planilha_registro_atendimentos.xlsx
+++ b/planilha_registro_atendimentos.xlsx
@@ -1730,8 +1730,8 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="D3">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
-      <formula>0</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>D3&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6:E110">
@@ -1869,8 +1869,8 @@
     <mergeCell ref="A13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
-      <formula>0</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>B6&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Corrige deficit para soma abaixo de 160 minutos
</commit_message>
<xml_diff>
--- a/planilha_registro_atendimentos.xlsx
+++ b/planilha_registro_atendimentos.xlsx
@@ -1731,7 +1731,7 @@
   </mergeCells>
   <conditionalFormatting sqref="D3">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>D3&lt;0</formula>
+      <formula>D3&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6:E110">
@@ -1870,7 +1870,7 @@
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>B6&lt;0</formula>
+      <formula>B6&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Destaca soma abaixo da previsao em vermelho
</commit_message>
<xml_diff>
--- a/planilha_registro_atendimentos.xlsx
+++ b/planilha_registro_atendimentos.xlsx
@@ -1734,8 +1734,13 @@
       <formula>D3&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>B3&lt;D2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A6:E110">
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="3" dxfId="1">
       <formula>$A6="Excepcional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1873,6 +1878,11 @@
       <formula>B6&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B5">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>B5&lt;B4</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Corrige calculo de deficit acima da previsao
</commit_message>
<xml_diff>
--- a/planilha_registro_atendimentos.xlsx
+++ b/planilha_registro_atendimentos.xlsx
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="D3" s="6">
-        <f>D2-B3</f>
+        <f>IF(B3&lt;D2,D2-B3,0)</f>
         <v/>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>4. O saldo é calculado por: previsão de atendimentos − soma de minutos. Saldo negativo aparece em vermelho.</t>
+          <t>4. O déficit mostra apenas os minutos faltantes: se a soma for menor que 160, calcula 160 − soma; se for igual ou maior, mostra 0.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Exibe credito e deficit com texto
</commit_message>
<xml_diff>
--- a/planilha_registro_atendimentos.xlsx
+++ b/planilha_registro_atendimentos.xlsx
@@ -19,10 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="0;[Red]-0;0"/>
-    <numFmt numFmtId="166" formatCode="hh:mm"/>
+    <numFmt numFmtId="165" formatCode="hh:mm"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -134,7 +133,7 @@
     <xf numFmtId="1" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,7 +142,7 @@
     <xf numFmtId="49" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -152,7 +151,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -168,7 +167,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -639,11 +638,11 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Saldo / déficit (minutos)</t>
+          <t>Resultado</t>
         </is>
       </c>
       <c r="D3" s="6">
-        <f>IF(B3&lt;D2,D2-B3,0)</f>
+        <f>IF(B3=0,"",IF(B3&lt;D2,"Déficit de "&amp;(D2-B3)&amp;" min",IF(B3&gt;D2,"Crédito de "&amp;(B3-D2)&amp;" min","Sem crédito ou déficit")))</f>
         <v/>
       </c>
     </row>
@@ -1731,16 +1730,11 @@
   </mergeCells>
   <conditionalFormatting sqref="D3">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>D3&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3">
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>B3&lt;D2</formula>
+      <formula>LEFT(D3,7)="Déficit"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6:E110">
-    <cfRule type="expression" priority="3" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="1">
       <formula>$A6="Excepcional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1822,7 +1816,7 @@
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Saldo / déficit</t>
+          <t>Resultado</t>
         </is>
       </c>
       <c r="B6" s="18">
@@ -1861,7 +1855,7 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>4. O déficit mostra apenas os minutos faltantes: se a soma for menor que 160, calcula 160 − soma; se for igual ou maior, mostra 0.</t>
+          <t>4. O resultado mostra “Déficit de X min” quando faltar tempo e “Crédito de X min” quando ultrapassar 160 minutos. Somente o déficit fica vermelho.</t>
         </is>
       </c>
     </row>
@@ -1875,12 +1869,7 @@
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>B6&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5">
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>B5&lt;B4</formula>
+      <formula>LEFT(B6,7)="Déficit"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>